<commit_message>
Add Agent Performance cases
</commit_message>
<xml_diff>
--- a/cypress/downloads/Agents_20251203.xlsx
+++ b/cypress/downloads/Agents_20251203.xlsx
@@ -35,7 +35,7 @@
     <t>Active</t>
   </si>
   <si>
-    <t>Motor Renewals Team (Cairo), Motor Renewals Team (Alexandria), Non-Motor Renewals Team (Cairo), Non-Motor Renewals Team (Alexandria), Medical &amp; Life Renewals Team (Cairo), Medical &amp; Life Renewals Team (Alexandria), Corporate Motor Renewals Team (Cairo), Corporate Motor Renewals Team (Alexandria), Corporate Non-Motor Renewals Team (Cairo), Corporate Non-Motor Renewals Team (Alexandria), Corporate Medical &amp; Life Renewals Team (Cairo), Corporate Medical &amp; Life Renewals Team (Alexandria), Claims Motor Team (Cairo), Claims Motor Team (Alexandria), Claims Non-Motor Team (Cairo), Claims Non-Motor Team (Alexandria), Claims Medical &amp; Life Team (Cairo), Claims Medical &amp; Life Team (Alexandria), Corporate Claims Motor Team (Cairo), Corporate Claims Motor Team (Alexandria), Corporate Claims Non-Motor Team (Cairo), Corporate Claims Non-Motor Team (Alexandria), Corporate Claims Medical &amp; Life Team (Cairo), Corporate Claims Medical &amp; Life Team (Alexandria), Motor New Sales Team, Non-Motor New Sales Team, Medical &amp; Life New Sales Team, Corporate Motor New Sales Team, Corporate Non-Motor New Sales Team, Corporate Medical &amp; Life New Sales Team, Request for support team, Desouky T, Desouky TU, Team 111111111111, Motor Renewals Team (Cairo) 2</t>
+    <t xml:space="preserve">Motor Renewals Team (Cairo) 99999999, Motor Renewals Team (Cairo)  865, Non-Motor Renewals Team (Cairo), Non-Motor Renewals Team (Alexandria), Medical &amp; Life Renewals Team (Cairo), Medical &amp; Life Renewals Team (Alexandria), Corporate Motor Renewals Team (Cairo), Corporate Motor Renewals Team (Alexandria), Corporate Non-Motor Renewals Team (Cairo), Corporate Non-Motor Renewals Team (Alexandria), Corporate Medical &amp; Life Renewals Team (Cairo), Corporate Medical &amp; Life Renewals Team (Alexandria), Claims Motor Team (Cairo), Claims Motor Team (Alexandria), Claims Non-Motor Team (Cairo), Claims Non-Motor Team (Alexandria), Claims Medical &amp; Life Team (Cairo), Claims Medical &amp; Life Team (Alexandria), Corporate Claims Motor Team (Cairo), Corporate Claims Motor Team (Alexandria), Corporate Claims Non-Motor Team (Cairo), Corporate Claims Non-Motor Team (Alexandria), Corporate Claims Medical &amp; Life Team (Cairo), Corporate Claims Medical &amp; Life Team (Alexandria), Motor New Sales Team, Non-Motor New Sales Team, Medical &amp; Life New Sales Team, Corporate Motor New Sales Team, Corporate Non-Motor New Sales Team, Corporate Medical &amp; Life New Sales Team, Request for support team, Motor Renewals Team (Cairo)  589, Motor Renewals Team (Cairo)  197, Motor Renewals Team (Cairo)  206, Motor Renewals Team (Cairo) 2</t>
   </si>
   <si>
     <t xml:space="preserve">Desouky  644</t>
@@ -143,7 +143,7 @@
     <t>119_Desouky@ntchnco.com</t>
   </si>
   <si>
-    <t>Motor Renewals Team (Cairo)</t>
+    <t>Motor Renewals Team (Cairo) 99999999</t>
   </si>
   <si>
     <t>May Mohamed</t>

</xml_diff>